<commit_message>
dataset updates, theme updates
</commit_message>
<xml_diff>
--- a/BACK-END/addon_details.xlsx
+++ b/BACK-END/addon_details.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C53"/>
+  <dimension ref="A1:C56"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -982,9 +982,42 @@
         <v>91</v>
       </c>
     </row>
+    <row r="54">
+      <c r="A54" t="str">
+        <v>KIM</v>
+      </c>
+      <c r="B54" t="str">
+        <v>Integrated business planning, Demand supply alignment, Capacity management</v>
+      </c>
+      <c r="C54" t="str">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="str">
+        <v>TOKN</v>
+      </c>
+      <c r="B55" t="str">
+        <v>Conditional orders, Automated trading, Risk management</v>
+      </c>
+      <c r="C55" t="str">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="str">
+        <v>SolBox SmartMove</v>
+      </c>
+      <c r="B56" t="str">
+        <v>Time tracking, Employee attendance, Payroll integration</v>
+      </c>
+      <c r="C56" t="str">
+        <v>55</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C53"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C56"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
myob replaced to bitzify
</commit_message>
<xml_diff>
--- a/BACK-END/addon_details.xlsx
+++ b/BACK-END/addon_details.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C56"/>
+  <dimension ref="A1:C59"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1015,9 +1015,42 @@
         <v>55</v>
       </c>
     </row>
+    <row r="57">
+      <c r="A57" t="str">
+        <v>Buildlogic</v>
+      </c>
+      <c r="B57" t="str">
+        <v>Construction BI, Job forecasting, WIP management</v>
+      </c>
+      <c r="C57" t="str">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="str">
+        <v>biotime</v>
+      </c>
+      <c r="B58" t="str">
+        <v>Form integration, Data capture, Workflow automation</v>
+      </c>
+      <c r="C58" t="str">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="str">
+        <v>Autodesk Construction Cloud</v>
+      </c>
+      <c r="B59" t="str">
+        <v>Payroll processing, Employee management, Tax compliance</v>
+      </c>
+      <c r="C59" t="str">
+        <v>40</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C56"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C59"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>